<commit_message>
Widen the sample with global ODM peers
Adding more Korean cosmetics names cannot help much: their residuals
correlate 0.39, so the average beta's standard error bottoms out at
0.143 (0.147 even with 30 peers). Peers with a different common factor
can, so the sample now includes Intercos (IT) and Qingsong/Nox Bellcow
(CN), each measured against its home index and unlevered at its local
tax rate.

Result: mean residual correlation 0.40 → 0.26, SE 0.162 → 0.129, band
0.55–0.97 → 0.59–0.93. The unlevered medians of the global peers (0.56,
0.81) bracket the Korean median (0.670), which cross-checks it.

Nihon Shikizai is excluded by a screen fixed before looking at results
(D/E > 200% or market cap < 100bn KRW); including it would move the
median to 0.646, and the README says so.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/peer_beta.xlsx
+++ b/output/peer_beta.xlsx
@@ -11,11 +11,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="주간수익률" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추정오차" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="범위" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="회귀통계" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="이동베타" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="반도체비중" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터대조" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="부채매핑" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="확장표본" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="회귀통계" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="이동베타" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="반도체비중" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터대조" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="부채매핑" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1190,6 +1191,1151 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>account_id</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>account_nm</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>금액(억원)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>192820</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>코스맥스</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ifrs-full_CashAndCashEquivalents</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>현금및현금성자산</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="n">
+        <v>3367.26180991</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>192820</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>코스맥스</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>financial_aggregate</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ifrs-full_CurrentFinancialLiabilities</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>단기금융부채</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="n">
+        <v>9010.01524807</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>192820</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>코스맥스</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>financial_aggregate</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ifrs-full_NoncurrentFinancialLiabilities</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>장기금융부채</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>3713.39626648</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>161890</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>한국콜마</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ifrs-full_CurrentBondsIssuedAndCurrentPortionOfNoncurrentBondsIssued</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>유동사채</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>1468.84324371</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>161890</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>한국콜마</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ifrs-full_CurrentLoansReceivedAndCurrentPortionOfNoncurrentLoansReceived</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>단기차입금</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>6647.81055354</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>161890</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>한국콜마</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ifrs-full_NoncurrentPortionOfNoncurrentBondsIssued</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>비유동사채</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>2086.3987761</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>161890</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>한국콜마</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ifrs-full_NoncurrentPortionOfNoncurrentLoansReceived</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>장기차입금</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>1610.37269682</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>161890</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>한국콜마</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>lease</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ifrs-full_CurrentLeaseLiabilities</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>유동리스부채</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>147.71505336</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>161890</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>한국콜마</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>lease</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ifrs-full_NoncurrentLeaseLiabilities</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>비유동리스부채</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>413.08771925</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>161890</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>한국콜마</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ifrs-full_CashAndCashEquivalents</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>현금및현금성자산</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>1768.17079758</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>241710</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>코스메카코리아</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ifrs-full_CurrentPortionOfLongtermBorrowings</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>유동성장기부채</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>77.64480278000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>241710</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>코스메카코리아</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ifrs-full_ShorttermBorrowings</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>단기차입금</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>1596.84810637</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>241710</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>코스메카코리아</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ifrs-full_LongtermBorrowings</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>장기차입금</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>583.73069911</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>241710</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>코스메카코리아</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>lease</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ifrs-full_CurrentLeaseLiabilities</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>리스유동부채</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>25.84860068</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>241710</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>코스메카코리아</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>lease</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ifrs-full_NoncurrentLeaseLiabilities</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>리스비유동부채</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>45.60761931</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>241710</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>코스메카코리아</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ifrs-full_CashAndCashEquivalents</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>현금및현금성자산</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>774.5964797399999</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>352480</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>씨앤씨인터내셔널</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>dart_CurrentLoansReceived</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>단기차입금</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>119.7998</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>352480</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>씨앤씨인터내셔널</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>dart_CurrentPortionOfConvertibleBonds</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>전환사채(유동)</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>352480</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>씨앤씨인터내셔널</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>dart_CurrentPortionOfNoncurrentLoansReceived</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>유동성장기부채</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>352480</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>씨앤씨인터내셔널</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>lease</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ifrs-full_CurrentLeaseLiabilities</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>리스부채(유동)</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>21.00096633</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>352480</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>씨앤씨인터내셔널</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>lease</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ifrs-full_NoncurrentLeaseLiabilities</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>리스부채(비유동)</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>17.08797644</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>352480</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>씨앤씨인터내셔널</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ifrs-full_CashAndCashEquivalents</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>현금및현금성자산</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>1191.7419076</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>950140</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>잉글우드랩</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>-표준계정코드 미사용-</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>유동성장기부채</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>0.00419332</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>950140</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>잉글우드랩</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>-표준계정코드 미사용-</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>단기차입금</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="n">
+        <v>0.09082063</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>950140</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>잉글우드랩</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>-표준계정코드 미사용-</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>장기차입금</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>0.01145287</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>950140</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>잉글우드랩</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>lease</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>-표준계정코드 미사용-</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>리스부채</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>0.00785215</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>950140</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>잉글우드랩</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>lease</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>-표준계정코드 미사용-</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>리스부채</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="n">
+        <v>0.02448415</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>950140</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>잉글우드랩</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ifrs-full_CashAndCashEquivalents</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>현금및현금성자산</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="n">
+        <v>0.29045839</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>003350</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>한국화장품제조</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ifrs-full_ShorttermBorrowings</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>단기차입부채</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>003350</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>한국화장품제조</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>borrowings</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>dart_ExchangeableBonds</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>교환사채</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="n">
+        <v>555.30033026</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>003350</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>한국화장품제조</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ifrs-full_CashAndCashEquivalents</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>현금및현금성자산</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>620.19862427</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4699,6 +5845,259 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>해외 ODM 을 더한 확장표본 — 공통요인이 다른 표본을 넣어야 추정오차가 실제로 줄어든다</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>회사</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>국가</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>시장지수</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>원시 β</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>R²</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>D/E</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>βu</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>통화</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>재무제표 기준일</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Intercos</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>이탈리아</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FTSEMIB.MI</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>0.4691769507693567</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>0.1534220931747355</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>0.0839846840951568</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>0.2128358092894584</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>0.5586249746476299</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>青松股份(노스벨)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>399001.SZ</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>0.7730490204716446</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0.1394552602296274</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0.2315151459583877</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0.06885638044327268</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0.8063034888787709</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>국내 6사</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>확장표본 8사</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>평균 베타의 표준오차</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>0.1615402136955219</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>0.1290286202608871</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>잔차 간 평균 상관</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>0.4007825071363929</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>0.2585932709175009</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>βu 중앙값</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>0.6703914537602538</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>0.6703914537602538</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>재레버 베타 구간 하한</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>0.5494102871092812</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>0.5898537275818528</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>재레버 베타 구간 상한</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>0.9663693278045949</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>0.9267329847673851</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>사전 스크리닝 제외: 日本色材工業研究所 (D/E 415% &gt; 기준 200%; 시가총액 210억원 &lt; 기준 1,000억원)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10764,7 +12163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15367,7 +16766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17701,7 +19100,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18245,1149 +19644,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>currency</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>line</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>account_id</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>account_nm</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>금액(억원)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>192820</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>코스맥스</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>ifrs-full_CashAndCashEquivalents</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>현금및현금성자산</t>
-        </is>
-      </c>
-      <c r="G2" s="10" t="n">
-        <v>3367.26180991</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>192820</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>코스맥스</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>financial_aggregate</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>ifrs-full_CurrentFinancialLiabilities</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>단기금융부채</t>
-        </is>
-      </c>
-      <c r="G3" s="10" t="n">
-        <v>9010.01524807</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>192820</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>코스맥스</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>financial_aggregate</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>ifrs-full_NoncurrentFinancialLiabilities</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>장기금융부채</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="n">
-        <v>3713.39626648</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>161890</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>한국콜마</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>ifrs-full_CurrentBondsIssuedAndCurrentPortionOfNoncurrentBondsIssued</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>유동사채</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="n">
-        <v>1468.84324371</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>161890</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>한국콜마</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>ifrs-full_CurrentLoansReceivedAndCurrentPortionOfNoncurrentLoansReceived</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>단기차입금</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>6647.81055354</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>161890</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>한국콜마</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>ifrs-full_NoncurrentPortionOfNoncurrentBondsIssued</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>비유동사채</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>2086.3987761</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>161890</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>한국콜마</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>ifrs-full_NoncurrentPortionOfNoncurrentLoansReceived</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>장기차입금</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>1610.37269682</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>161890</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>한국콜마</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>lease</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>ifrs-full_CurrentLeaseLiabilities</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>유동리스부채</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>147.71505336</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>161890</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>한국콜마</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>lease</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>ifrs-full_NoncurrentLeaseLiabilities</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>비유동리스부채</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>413.08771925</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>161890</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>한국콜마</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>ifrs-full_CashAndCashEquivalents</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>현금및현금성자산</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="n">
-        <v>1768.17079758</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>241710</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>코스메카코리아</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>ifrs-full_CurrentPortionOfLongtermBorrowings</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>유동성장기부채</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="n">
-        <v>77.64480278000001</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>241710</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>코스메카코리아</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>ifrs-full_ShorttermBorrowings</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>단기차입금</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="n">
-        <v>1596.84810637</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>241710</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>코스메카코리아</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>ifrs-full_LongtermBorrowings</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>장기차입금</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="n">
-        <v>583.73069911</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>241710</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>코스메카코리아</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>lease</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>ifrs-full_CurrentLeaseLiabilities</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>리스유동부채</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="n">
-        <v>25.84860068</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>241710</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>코스메카코리아</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>lease</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>ifrs-full_NoncurrentLeaseLiabilities</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>리스비유동부채</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="n">
-        <v>45.60761931</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>241710</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>코스메카코리아</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>ifrs-full_CashAndCashEquivalents</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>현금및현금성자산</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="n">
-        <v>774.5964797399999</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>352480</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>씨앤씨인터내셔널</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>dart_CurrentLoansReceived</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>단기차입금</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>119.7998</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>352480</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>씨앤씨인터내셔널</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>dart_CurrentPortionOfConvertibleBonds</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>전환사채(유동)</t>
-        </is>
-      </c>
-      <c r="G19" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>352480</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>씨앤씨인터내셔널</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>dart_CurrentPortionOfNoncurrentLoansReceived</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>유동성장기부채</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>352480</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>씨앤씨인터내셔널</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>lease</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>ifrs-full_CurrentLeaseLiabilities</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>리스부채(유동)</t>
-        </is>
-      </c>
-      <c r="G21" s="10" t="n">
-        <v>21.00096633</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>352480</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>씨앤씨인터내셔널</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>lease</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>ifrs-full_NoncurrentLeaseLiabilities</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>리스부채(비유동)</t>
-        </is>
-      </c>
-      <c r="G22" s="10" t="n">
-        <v>17.08797644</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>352480</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>씨앤씨인터내셔널</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>ifrs-full_CashAndCashEquivalents</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>현금및현금성자산</t>
-        </is>
-      </c>
-      <c r="G23" s="10" t="n">
-        <v>1191.7419076</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>950140</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>잉글우드랩</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>-표준계정코드 미사용-</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>유동성장기부채</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="n">
-        <v>0.00419332</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>950140</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>잉글우드랩</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>-표준계정코드 미사용-</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>단기차입금</t>
-        </is>
-      </c>
-      <c r="G25" s="10" t="n">
-        <v>0.09082063</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>950140</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>잉글우드랩</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>-표준계정코드 미사용-</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>장기차입금</t>
-        </is>
-      </c>
-      <c r="G26" s="10" t="n">
-        <v>0.01145287</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>950140</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>잉글우드랩</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>lease</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>-표준계정코드 미사용-</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>리스부채</t>
-        </is>
-      </c>
-      <c r="G27" s="10" t="n">
-        <v>0.00785215</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>950140</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>잉글우드랩</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>lease</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>-표준계정코드 미사용-</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>리스부채</t>
-        </is>
-      </c>
-      <c r="G28" s="10" t="n">
-        <v>0.02448415</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>950140</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>잉글우드랩</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>ifrs-full_CashAndCashEquivalents</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>현금및현금성자산</t>
-        </is>
-      </c>
-      <c r="G29" s="10" t="n">
-        <v>0.29045839</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>003350</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>한국화장품제조</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ifrs-full_ShorttermBorrowings</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>단기차입부채</t>
-        </is>
-      </c>
-      <c r="G30" s="10" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>003350</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>한국화장품제조</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>borrowings</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>dart_ExchangeableBonds</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>교환사채</t>
-        </is>
-      </c>
-      <c r="G31" s="10" t="n">
-        <v>555.30033026</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>003350</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>한국화장품제조</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>ifrs-full_CashAndCashEquivalents</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>현금및현금성자산</t>
-        </is>
-      </c>
-      <c r="G32" s="10" t="n">
-        <v>620.19862427</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>